<commit_message>
add timeliness charts for Article IV and Program reports
- Generated big-grid timeliness charts for bondholders and china,
  using Article IV Reports and Program Reports as mention sources
  (separate from DSA analysis).
- Generated gap histograms with outliers excluded:
  - Bondholders × Article IV: Congo Rep, Lao PDR
  - Bondholders × Program: Ethiopia, Congo Rep
  - China × Article IV: St. Vincent, Grenada, Lesotho
  - China × Program: Grenada
- Embedded histograms into timeliness Excel files (Gap Histogram
  sheets).
- Removed obsolete DSA histograms with outliers.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/timeliness/timeliness_bondholders_aiv.xlsx
+++ b/outputs/timeliness/timeliness_bondholders_aiv.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Time Series" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap Histogram" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -124,6 +125,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="5143500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -21778,4 +21809,18 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>